<commit_message>
Including classes for ports (locations) loading and historical weather data (meteorologia)
</commit_message>
<xml_diff>
--- a/data/raw/porto/porto.xlsx
+++ b/data/raw/porto/porto.xlsx
@@ -5,18 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Graduação e Pós\USP\MBA USP IA e Big Data\TCC\port_leadtime_prediction\data\raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Graduação e Pós\USP\MBA USP IA e Big Data\TCC\port_leadtime_prediction\data\raw\porto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C3C7855-C32C-43BC-BD87-418B66548B97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4986D6D2-AE6E-46E5-B9DA-46EE7F484D2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4590" yWindow="4590" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portos" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Portos!$A$1:$D$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Portos!$A$1:$G$126</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="335">
   <si>
     <t>BRSSZ</t>
   </si>
@@ -338,9 +338,6 @@
     <t>TERMINAL PORTUÁRIO FLUVIAL - COPESUL</t>
   </si>
   <si>
-    <t>SANTA CLARA</t>
-  </si>
-  <si>
     <t>RS</t>
   </si>
   <si>
@@ -1023,6 +1020,30 @@
   </si>
   <si>
     <t>CARAVELAS</t>
+  </si>
+  <si>
+    <t>NORDESTE</t>
+  </si>
+  <si>
+    <t>NORTE</t>
+  </si>
+  <si>
+    <t>REGIAO</t>
+  </si>
+  <si>
+    <t>SUDESTE</t>
+  </si>
+  <si>
+    <t>SUL</t>
+  </si>
+  <si>
+    <t>TRIUNFO</t>
+  </si>
+  <si>
+    <t>LATITUDE</t>
+  </si>
+  <si>
+    <t>LONGITUDE</t>
   </si>
 </sst>
 </file>
@@ -1275,16 +1296,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D126"/>
+  <dimension ref="A1:G126"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
-    <col min="2" max="2" width="57.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="61.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>91</v>
       </c>
@@ -1297,8 +1320,17 @@
       <c r="D1" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" t="s">
+        <v>329</v>
+      </c>
+      <c r="F1" t="s">
+        <v>333</v>
+      </c>
+      <c r="G1" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>57</v>
       </c>
@@ -1311,8 +1343,17 @@
       <c r="D2" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>328</v>
+      </c>
+      <c r="F2">
+        <v>-2.1737820000000001</v>
+      </c>
+      <c r="G2" s="1">
+        <v>-56.105980000000002</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>49</v>
       </c>
@@ -1320,1736 +1361,2852 @@
         <v>98</v>
       </c>
       <c r="C3" t="s">
+        <v>332</v>
+      </c>
+      <c r="D3" t="s">
         <v>99</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
+        <v>331</v>
+      </c>
+      <c r="F3" s="1">
+        <v>-29.948609999999999</v>
+      </c>
+      <c r="G3" s="1">
+        <v>-51.623888000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
         <v>101</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>102</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>103</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>327</v>
+      </c>
+      <c r="F4" s="1">
+        <v>-5.1063868624376898</v>
+      </c>
+      <c r="G4" s="1">
+        <v>-36.317917702612</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>105</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>106</v>
       </c>
-      <c r="C5" t="s">
-        <v>107</v>
-      </c>
       <c r="D5" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F5" s="1">
+        <v>-29.931204205870799</v>
+      </c>
+      <c r="G5" s="1">
+        <v>-51.2827810587576</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>50</v>
       </c>
       <c r="B6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C6" t="s">
         <v>108</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>109</v>
       </c>
-      <c r="D6" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6" t="s">
+        <v>330</v>
+      </c>
+      <c r="F6" s="1">
+        <v>-21.814444000000002</v>
+      </c>
+      <c r="G6" s="1">
+        <v>-40.998333000000002</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
       <c r="B7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C7" t="s">
         <v>111</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>112</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
+        <v>327</v>
+      </c>
+      <c r="F7" s="1">
+        <v>-16.03</v>
+      </c>
+      <c r="G7" s="1">
+        <v>-38.923749000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B8" t="s">
         <v>114</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>115</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
+        <v>109</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F8" s="1">
+        <v>-23</v>
+      </c>
+      <c r="G8" s="1">
+        <v>-44.247222000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>116</v>
       </c>
-      <c r="D8" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
         <v>117</v>
       </c>
-      <c r="B9" t="s">
-        <v>118</v>
-      </c>
       <c r="C9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D9" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F9" s="1">
+        <v>-23.061388000000001</v>
+      </c>
+      <c r="G9" s="1">
+        <v>-44.228889000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>55</v>
       </c>
       <c r="B10" t="s">
+        <v>118</v>
+      </c>
+      <c r="C10" t="s">
+        <v>115</v>
+      </c>
+      <c r="D10" t="s">
+        <v>109</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F10" s="1">
+        <v>-23.01183</v>
+      </c>
+      <c r="G10" s="1">
+        <v>-44.310650000000003</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>119</v>
       </c>
-      <c r="C10" t="s">
-        <v>116</v>
-      </c>
-      <c r="D10" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="B11" t="s">
         <v>120</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>121</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>122</v>
       </c>
-      <c r="D11" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E11" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F11" s="1">
+        <v>-10.843889000000001</v>
+      </c>
+      <c r="G11" s="1">
+        <v>-36.919167000000002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>36</v>
       </c>
       <c r="B12" t="s">
+        <v>123</v>
+      </c>
+      <c r="C12" t="s">
         <v>124</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>125</v>
       </c>
-      <c r="D12" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E12" t="s">
+        <v>327</v>
+      </c>
+      <c r="F12" s="1">
+        <v>-2.6783320000000002</v>
+      </c>
+      <c r="G12" s="1">
+        <v>-44.360556000000003</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
       <c r="B13" t="s">
+        <v>126</v>
+      </c>
+      <c r="C13" t="s">
         <v>127</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>128</v>
       </c>
-      <c r="D13" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E13" t="s">
+        <v>331</v>
+      </c>
+      <c r="F13" s="1">
+        <v>-25.44166666666667</v>
+      </c>
+      <c r="G13" s="1">
+        <v>-48.691666666666663</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>47</v>
       </c>
       <c r="B14" t="s">
+        <v>129</v>
+      </c>
+      <c r="C14" t="s">
         <v>130</v>
       </c>
-      <c r="C14" t="s">
-        <v>131</v>
-      </c>
       <c r="D14" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F14" s="1">
+        <v>-12.783056</v>
+      </c>
+      <c r="G14" s="1">
+        <v>-38.476388</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>27</v>
       </c>
       <c r="B15" t="s">
+        <v>131</v>
+      </c>
+      <c r="C15" t="s">
         <v>132</v>
       </c>
-      <c r="C15" t="s">
-        <v>133</v>
-      </c>
       <c r="D15" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F15" s="1">
+        <v>-12.753888</v>
+      </c>
+      <c r="G15" s="1">
+        <v>-38.624305</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>82</v>
       </c>
       <c r="B16" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C16" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D16" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F16" s="1">
+        <v>-12.812222</v>
+      </c>
+      <c r="G16" s="1">
+        <v>-38.663333000000002</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>9</v>
       </c>
       <c r="B17" t="s">
+        <v>134</v>
+      </c>
+      <c r="C17" t="s">
         <v>135</v>
       </c>
-      <c r="C17" t="s">
-        <v>136</v>
-      </c>
       <c r="D17" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F17" s="1">
+        <v>-12.783333000000001</v>
+      </c>
+      <c r="G17" s="1">
+        <v>-38.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>4</v>
       </c>
       <c r="B18" t="s">
+        <v>136</v>
+      </c>
+      <c r="C18" t="s">
         <v>137</v>
       </c>
-      <c r="C18" t="s">
-        <v>138</v>
-      </c>
       <c r="D18" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+        <v>103</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F18" s="1">
+        <v>-4.8183333333333334</v>
+      </c>
+      <c r="G18" s="1">
+        <v>-37.045277777777777</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>72</v>
       </c>
       <c r="B19" t="s">
+        <v>138</v>
+      </c>
+      <c r="C19" t="s">
+        <v>121</v>
+      </c>
+      <c r="D19" t="s">
+        <v>122</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F19" s="1">
+        <v>-10.843889000000001</v>
+      </c>
+      <c r="G19" s="1">
+        <v>-36.919167000000002</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>139</v>
       </c>
-      <c r="C19" t="s">
-        <v>122</v>
-      </c>
-      <c r="D19" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="B20" t="s">
         <v>140</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>141</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>142</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F20" s="1">
+        <v>-26.883054999999999</v>
+      </c>
+      <c r="G20" s="1">
+        <v>-48.673611000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="B21" t="s">
         <v>144</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>145</v>
-      </c>
-      <c r="C21" t="s">
-        <v>146</v>
       </c>
       <c r="D21" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E21" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F21" s="1">
+        <v>-1.3561110000000001</v>
+      </c>
+      <c r="G21" s="1">
+        <v>-48.481389</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>56</v>
       </c>
       <c r="B22" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C22" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D22" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E22" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F22" s="1">
+        <v>-1.4422219999999999</v>
+      </c>
+      <c r="G22" s="1">
+        <v>-48.496110999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>38</v>
       </c>
       <c r="B23" t="s">
+        <v>147</v>
+      </c>
+      <c r="C23" t="s">
         <v>148</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>149</v>
       </c>
-      <c r="D23" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E23" t="s">
+        <v>327</v>
+      </c>
+      <c r="F23" s="1">
+        <v>-6.97161039716618</v>
+      </c>
+      <c r="G23" s="1">
+        <v>-34.838534308256101</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>21</v>
       </c>
       <c r="B24" t="s">
+        <v>150</v>
+      </c>
+      <c r="C24" t="s">
         <v>151</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>152</v>
       </c>
-      <c r="D24" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E24" t="s">
+        <v>327</v>
+      </c>
+      <c r="F24" s="1">
+        <v>-3.7213980000000002</v>
+      </c>
+      <c r="G24" s="1">
+        <v>-38.520544999999998</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>29</v>
       </c>
       <c r="B25" t="s">
+        <v>153</v>
+      </c>
+      <c r="C25" t="s">
         <v>154</v>
       </c>
-      <c r="C25" t="s">
-        <v>155</v>
-      </c>
       <c r="D25" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F25" s="1">
+        <v>-28.228888000000001</v>
+      </c>
+      <c r="G25" s="1">
+        <v>-48.658056000000002</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>53</v>
       </c>
       <c r="B26" t="s">
+        <v>155</v>
+      </c>
+      <c r="C26" t="s">
         <v>156</v>
       </c>
-      <c r="C26" t="s">
-        <v>157</v>
-      </c>
       <c r="D26" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F26" s="1">
+        <v>-23.013331999999998</v>
+      </c>
+      <c r="G26" s="1">
+        <v>-44.033332000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>61</v>
       </c>
       <c r="B27" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F27" s="1">
+        <v>-22.933150000000001</v>
+      </c>
+      <c r="G27" s="1">
+        <v>-43.837310000000002</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>59</v>
       </c>
       <c r="B28" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F28" s="1">
+        <v>-22.925000000000001</v>
+      </c>
+      <c r="G28" s="1">
+        <v>-43.852221</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>10</v>
       </c>
       <c r="B29" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F29" s="1">
+        <v>-22.933150000000001</v>
+      </c>
+      <c r="G29" s="1">
+        <v>-43.837310000000002</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>35</v>
       </c>
       <c r="B30" t="s">
+        <v>160</v>
+      </c>
+      <c r="C30" t="s">
         <v>161</v>
       </c>
-      <c r="C30" t="s">
-        <v>162</v>
-      </c>
       <c r="D30" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F30" s="1">
+        <v>-26.182915999999999</v>
+      </c>
+      <c r="G30" s="1">
+        <v>-48.606138000000001</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>80</v>
       </c>
       <c r="B31" t="s">
+        <v>162</v>
+      </c>
+      <c r="C31" t="s">
         <v>163</v>
       </c>
-      <c r="C31" t="s">
-        <v>164</v>
-      </c>
       <c r="D31" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F31" s="1">
+        <v>-14.780521999999999</v>
+      </c>
+      <c r="G31" s="1">
+        <v>-39.026533000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>41</v>
       </c>
       <c r="B32" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C32" t="s">
+        <v>124</v>
+      </c>
+      <c r="D32" t="s">
         <v>125</v>
       </c>
-      <c r="D32" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E32" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F32" s="1">
+        <v>-2.5750000000000002</v>
+      </c>
+      <c r="G32" s="1">
+        <v>-44.37</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>37</v>
       </c>
       <c r="B33" t="s">
+        <v>165</v>
+      </c>
+      <c r="C33" t="s">
         <v>166</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>167</v>
       </c>
-      <c r="D33" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E33" t="s">
+        <v>328</v>
+      </c>
+      <c r="F33" s="1">
+        <v>-3.1361110000000001</v>
+      </c>
+      <c r="G33" s="1">
+        <v>-58.483611000000003</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>74</v>
       </c>
       <c r="B34" t="s">
+        <v>168</v>
+      </c>
+      <c r="C34" t="s">
+        <v>166</v>
+      </c>
+      <c r="D34" t="s">
+        <v>167</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F34" s="1">
+        <v>-3.1361110000000001</v>
+      </c>
+      <c r="G34" s="1">
+        <v>-58.483611000000003</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>169</v>
       </c>
-      <c r="C34" t="s">
+      <c r="B35" t="s">
+        <v>170</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="D34" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>170</v>
-      </c>
-      <c r="B35" t="s">
+      <c r="E35" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F35" s="1">
+        <v>-3.2292000000000001</v>
+      </c>
+      <c r="G35" s="1">
+        <v>-59.000008000000001</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>171</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="B36" t="s">
+        <v>172</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="D36" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="D35" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>172</v>
-      </c>
-      <c r="B36" t="s">
-        <v>173</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E36" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F36" s="1">
+        <v>-3.2292000000000001</v>
+      </c>
+      <c r="G36" s="1">
+        <v>-59.000008000000001</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>70</v>
       </c>
       <c r="B37" t="s">
+        <v>173</v>
+      </c>
+      <c r="C37" t="s">
         <v>174</v>
       </c>
-      <c r="C37" t="s">
-        <v>175</v>
-      </c>
       <c r="D37" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F37" s="1">
+        <v>-26.897220999999998</v>
+      </c>
+      <c r="G37" s="1">
+        <v>-48.670278000000003</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>76</v>
       </c>
       <c r="B38" t="s">
+        <v>175</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F38" s="1">
+        <v>-26.876667000000008</v>
+      </c>
+      <c r="G38" s="1">
+        <v>-48.711387999999999</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>176</v>
       </c>
-      <c r="C38" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+      <c r="B39" t="s">
         <v>177</v>
       </c>
-      <c r="B39" t="s">
-        <v>178</v>
-      </c>
       <c r="C39" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F39" s="1">
+        <v>-26.888055000000001</v>
+      </c>
+      <c r="G39" s="1">
+        <v>-48.683889000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>79</v>
       </c>
       <c r="B40" t="s">
+        <v>178</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F40" s="1">
+        <v>-26.883054999999999</v>
+      </c>
+      <c r="G40" s="1">
+        <v>-48.673610999999987</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>179</v>
       </c>
-      <c r="C40" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+      <c r="B41" t="s">
         <v>180</v>
       </c>
-      <c r="B41" t="s">
+      <c r="C41" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F41" s="1">
+        <v>-26.883054999999999</v>
+      </c>
+      <c r="G41" s="1">
+        <v>-48.673611000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>181</v>
       </c>
-      <c r="C41" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+      <c r="B42" t="s">
         <v>182</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F42" s="1">
+        <v>-26.897220999999998</v>
+      </c>
+      <c r="G42" s="1">
+        <v>-48.670278000000003</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>183</v>
       </c>
-      <c r="C42" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+      <c r="B43" t="s">
         <v>184</v>
       </c>
-      <c r="B43" t="s">
-        <v>185</v>
-      </c>
       <c r="C43" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F43" s="1">
+        <v>-26.888055000000001</v>
+      </c>
+      <c r="G43" s="1">
+        <v>-48.683889000000001</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C44" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D44" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F44" s="1">
+        <v>-26.941666999999999</v>
+      </c>
+      <c r="G44" s="1">
+        <v>-48.5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>69</v>
       </c>
       <c r="B45" t="s">
+        <v>186</v>
+      </c>
+      <c r="C45" t="s">
         <v>187</v>
       </c>
-      <c r="C45" t="s">
-        <v>188</v>
-      </c>
       <c r="D45" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F45" s="1">
+        <v>-3.1355550000000001</v>
+      </c>
+      <c r="G45" s="1">
+        <v>-59.938333000000007</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>64</v>
       </c>
       <c r="B46" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F46" s="1">
+        <v>-3.1569440000000002</v>
+      </c>
+      <c r="G46" s="1">
+        <v>-59.998609999999992</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>90</v>
       </c>
       <c r="B47" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F47" s="1">
+        <v>-3.1497220000000001</v>
+      </c>
+      <c r="G47" s="1">
+        <v>-59.951667</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>67</v>
       </c>
       <c r="B48" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F48" s="1">
+        <v>-3.16</v>
+      </c>
+      <c r="G48" s="1">
+        <v>-59.991109999999999</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>81</v>
       </c>
       <c r="B49" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F49" s="1">
+        <v>-3.1227770000000001</v>
+      </c>
+      <c r="G49" s="1">
+        <v>-59.923610999999987</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>7</v>
       </c>
       <c r="B50" t="s">
+        <v>192</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F50" s="1">
+        <v>-3.1536360000000001</v>
+      </c>
+      <c r="G50" s="1">
+        <v>-60.000067000000001</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
         <v>193</v>
       </c>
-      <c r="C50" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+      <c r="B51" t="s">
         <v>194</v>
       </c>
-      <c r="B51" t="s">
+      <c r="C51" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F51" s="1">
+        <v>-3.1497220000000001</v>
+      </c>
+      <c r="G51" s="1">
+        <v>-59.951667</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>195</v>
       </c>
-      <c r="C51" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+      <c r="B52" t="s">
         <v>196</v>
       </c>
-      <c r="B52" t="s">
-        <v>197</v>
-      </c>
       <c r="C52" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F52" s="1">
+        <v>-3.1341666666666672</v>
+      </c>
+      <c r="G52" s="1">
+        <v>-60.029444444444437</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>78</v>
       </c>
       <c r="B53" t="s">
+        <v>197</v>
+      </c>
+      <c r="C53" t="s">
         <v>198</v>
       </c>
-      <c r="C53" t="s">
+      <c r="D53" t="s">
         <v>199</v>
       </c>
-      <c r="D53" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E53" t="s">
+        <v>328</v>
+      </c>
+      <c r="F53" s="1">
+        <v>-6.8333000000000005E-2</v>
+      </c>
+      <c r="G53" s="1">
+        <v>-51.159998999999992</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>60</v>
       </c>
       <c r="B54" t="s">
+        <v>200</v>
+      </c>
+      <c r="C54" t="s">
         <v>201</v>
       </c>
-      <c r="C54" t="s">
+      <c r="D54" t="s">
         <v>202</v>
       </c>
-      <c r="D54" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E54" t="s">
+        <v>327</v>
+      </c>
+      <c r="F54" s="1">
+        <v>-9.6938890000000004</v>
+      </c>
+      <c r="G54" s="1">
+        <v>-35.759166</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>24</v>
       </c>
       <c r="B55" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C55" t="s">
+        <v>201</v>
+      </c>
+      <c r="D55" t="s">
         <v>202</v>
       </c>
-      <c r="D55" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E55" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F55" s="1">
+        <v>-9.6833329999999993</v>
+      </c>
+      <c r="G55" s="1">
+        <v>-35.716667000000001</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>2</v>
       </c>
       <c r="B56" t="s">
+        <v>204</v>
+      </c>
+      <c r="C56" t="s">
         <v>205</v>
       </c>
-      <c r="C56" t="s">
-        <v>206</v>
-      </c>
       <c r="D56" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F56" s="1">
+        <v>-22.385833000000002</v>
+      </c>
+      <c r="G56" s="1">
+        <v>-41.768332000000001</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>83</v>
       </c>
       <c r="B57" t="s">
+        <v>206</v>
+      </c>
+      <c r="C57" t="s">
         <v>207</v>
-      </c>
-      <c r="C57" t="s">
-        <v>208</v>
       </c>
       <c r="D57" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E57" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F57" s="1">
+        <v>-0.85830700000000004</v>
+      </c>
+      <c r="G57" s="1">
+        <v>-52.541353000000001</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>33</v>
       </c>
       <c r="B58" t="s">
+        <v>208</v>
+      </c>
+      <c r="C58" t="s">
         <v>209</v>
       </c>
-      <c r="C58" t="s">
-        <v>210</v>
-      </c>
       <c r="D58" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+        <v>103</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F58" s="1">
+        <v>-5.7733333333333334</v>
+      </c>
+      <c r="G58" s="1">
+        <v>-35.205555555555563</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>54</v>
       </c>
       <c r="B59" t="s">
+        <v>210</v>
+      </c>
+      <c r="C59" t="s">
         <v>211</v>
       </c>
-      <c r="C59" t="s">
-        <v>212</v>
-      </c>
       <c r="D59" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F59" s="1">
+        <v>-22.87886</v>
+      </c>
+      <c r="G59" s="1">
+        <v>-43.122019999999999</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>34</v>
       </c>
       <c r="B60" t="s">
+        <v>212</v>
+      </c>
+      <c r="C60" t="s">
         <v>213</v>
       </c>
-      <c r="C60" t="s">
+      <c r="D60" t="s">
+        <v>142</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F60" s="1">
+        <v>-26.897777000000001</v>
+      </c>
+      <c r="G60" s="1">
+        <v>-48.662221000000002</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
         <v>214</v>
       </c>
-      <c r="D60" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+      <c r="B61" t="s">
         <v>215</v>
       </c>
-      <c r="B61" t="s">
+      <c r="C61" t="s">
+        <v>213</v>
+      </c>
+      <c r="D61" t="s">
+        <v>142</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F61" s="1">
+        <v>-26.897777000000001</v>
+      </c>
+      <c r="G61" s="1">
+        <v>-48.662221000000002</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
         <v>216</v>
       </c>
-      <c r="C61" t="s">
-        <v>214</v>
-      </c>
-      <c r="D61" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+      <c r="B62" t="s">
         <v>217</v>
       </c>
-      <c r="B62" t="s">
+      <c r="C62" t="s">
         <v>218</v>
       </c>
-      <c r="C62" t="s">
-        <v>219</v>
-      </c>
       <c r="D62" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F62" s="1">
+        <v>-26.897777000000001</v>
+      </c>
+      <c r="G62" s="1">
+        <v>-48.662221000000002</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>12</v>
       </c>
       <c r="B63" t="s">
+        <v>219</v>
+      </c>
+      <c r="C63" t="s">
         <v>220</v>
       </c>
-      <c r="C63" t="s">
-        <v>221</v>
-      </c>
       <c r="D63" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+      <c r="E63" t="s">
+        <v>327</v>
+      </c>
+      <c r="F63" s="1">
+        <v>-3.5266670000000002</v>
+      </c>
+      <c r="G63" s="1">
+        <v>-38.796388</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>20</v>
       </c>
       <c r="B64" t="s">
+        <v>221</v>
+      </c>
+      <c r="C64" t="s">
         <v>222</v>
       </c>
-      <c r="C64" t="s">
-        <v>223</v>
-      </c>
       <c r="D64" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F64" s="1">
+        <v>-31.78222222222222</v>
+      </c>
+      <c r="G64" s="1">
+        <v>-52.31805555555556</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>31</v>
       </c>
       <c r="B65" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C65" t="s">
+        <v>124</v>
+      </c>
+      <c r="D65" t="s">
         <v>125</v>
       </c>
-      <c r="D65" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E65" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F65" s="1">
+        <v>-2.5619429999999999</v>
+      </c>
+      <c r="G65" s="1">
+        <v>-44.379167000000002</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>6</v>
       </c>
       <c r="B66" t="s">
+        <v>224</v>
+      </c>
+      <c r="C66" t="s">
         <v>225</v>
       </c>
-      <c r="C66" t="s">
-        <v>226</v>
-      </c>
       <c r="D66" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+      <c r="E66" t="s">
+        <v>331</v>
+      </c>
+      <c r="F66" s="1">
+        <v>-25.5</v>
+      </c>
+      <c r="G66" s="1">
+        <v>-48.516666999999998</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>25</v>
       </c>
       <c r="B67" t="s">
+        <v>226</v>
+      </c>
+      <c r="C67" t="s">
         <v>227</v>
       </c>
-      <c r="C67" t="s">
-        <v>228</v>
-      </c>
       <c r="D67" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F67" s="1">
+        <v>-30.00194444444444</v>
+      </c>
+      <c r="G67" s="1">
+        <v>-51.208611111111111</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>22</v>
       </c>
       <c r="B68" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C68" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D68" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F68" s="1">
+        <v>-30.00194444444444</v>
+      </c>
+      <c r="G68" s="1">
+        <v>-51.208611111111111</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>73</v>
       </c>
       <c r="B69" t="s">
+        <v>229</v>
+      </c>
+      <c r="C69" t="s">
         <v>230</v>
       </c>
-      <c r="C69" t="s">
+      <c r="D69" t="s">
+        <v>99</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F69" s="1">
+        <v>-29.967082000000001</v>
+      </c>
+      <c r="G69" s="1">
+        <v>-51.203749000000002</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
         <v>231</v>
       </c>
-      <c r="D69" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
+      <c r="B70" t="s">
         <v>232</v>
       </c>
-      <c r="B70" t="s">
+      <c r="C70" t="s">
+        <v>230</v>
+      </c>
+      <c r="D70" t="s">
+        <v>99</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F70" s="1">
+        <v>-29.967915999999999</v>
+      </c>
+      <c r="G70" s="1">
+        <v>-51.203611000000002</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
         <v>233</v>
       </c>
-      <c r="C70" t="s">
-        <v>231</v>
-      </c>
-      <c r="D70" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+      <c r="B71" t="s">
         <v>234</v>
       </c>
-      <c r="B71" t="s">
+      <c r="C71" t="s">
         <v>235</v>
       </c>
-      <c r="C71" t="s">
+      <c r="D71" t="s">
         <v>236</v>
       </c>
-      <c r="D71" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E71" t="s">
+        <v>330</v>
+      </c>
+      <c r="F71" s="1">
+        <v>-19.842500000000001</v>
+      </c>
+      <c r="G71" s="1">
+        <v>-40.0625</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>84</v>
       </c>
       <c r="B72" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C72" t="s">
+        <v>235</v>
+      </c>
+      <c r="D72" t="s">
         <v>236</v>
       </c>
-      <c r="D72" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E72" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F72" s="1">
+        <v>-19.840831999999999</v>
+      </c>
+      <c r="G72" s="1">
+        <v>-40.057499</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>5</v>
       </c>
       <c r="B73" t="s">
+        <v>238</v>
+      </c>
+      <c r="C73" t="s">
         <v>239</v>
       </c>
-      <c r="C73" t="s">
+      <c r="D73" t="s">
         <v>240</v>
       </c>
-      <c r="D73" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E73" t="s">
+        <v>327</v>
+      </c>
+      <c r="F73" s="1">
+        <v>-8.0611239999999995</v>
+      </c>
+      <c r="G73" s="1">
+        <v>-34.866733000000004</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>13</v>
       </c>
       <c r="B74" t="s">
+        <v>241</v>
+      </c>
+      <c r="C74" t="s">
         <v>242</v>
       </c>
-      <c r="C74" t="s">
-        <v>243</v>
-      </c>
       <c r="D74" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F74" s="1">
+        <v>-32.122222000000001</v>
+      </c>
+      <c r="G74" s="1">
+        <v>-52.093333000000001</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>3</v>
       </c>
       <c r="B75" t="s">
+        <v>243</v>
+      </c>
+      <c r="C75" t="s">
         <v>244</v>
       </c>
-      <c r="C75" t="s">
-        <v>245</v>
-      </c>
       <c r="D75" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F75" s="1">
+        <v>-22.891943999999999</v>
+      </c>
+      <c r="G75" s="1">
+        <v>-43.195278000000002</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>1</v>
       </c>
       <c r="B76" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C76" t="s">
+        <v>108</v>
+      </c>
+      <c r="D76" t="s">
         <v>109</v>
       </c>
-      <c r="D76" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E76" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F76" s="1">
+        <v>-21.814444000000002</v>
+      </c>
+      <c r="G76" s="1">
+        <v>-40.998333000000002</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>16</v>
       </c>
       <c r="B77" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C77" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D77" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F77" s="1">
+        <v>-29.916111000000001</v>
+      </c>
+      <c r="G77" s="1">
+        <v>-51.239722</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>58</v>
       </c>
       <c r="B78" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C78" t="s">
-        <v>212</v>
-      </c>
-      <c r="D78" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+        <v>211</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F78" s="1">
+        <v>-22.87886</v>
+      </c>
+      <c r="G78" s="1">
+        <v>-43.122019999999999</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>23</v>
       </c>
       <c r="B79" t="s">
+        <v>248</v>
+      </c>
+      <c r="C79" t="s">
         <v>249</v>
       </c>
-      <c r="C79" t="s">
-        <v>250</v>
-      </c>
       <c r="D79" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F79" s="1">
+        <v>-30.135833000000002</v>
+      </c>
+      <c r="G79" s="1">
+        <v>-51.310276999999999</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>66</v>
       </c>
       <c r="B80" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C80" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D80" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F80" s="1">
+        <v>-29.968471000000001</v>
+      </c>
+      <c r="G80" s="1">
+        <v>-51.182361000000007</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>26</v>
       </c>
       <c r="B81" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C81" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D81" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F81" s="1">
+        <v>-32.079720999999999</v>
+      </c>
+      <c r="G81" s="1">
+        <v>-52.094999000000008</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>88</v>
       </c>
       <c r="B82" t="s">
+        <v>252</v>
+      </c>
+      <c r="C82" t="s">
         <v>253</v>
       </c>
-      <c r="C82" t="s">
+      <c r="D82" t="s">
+        <v>122</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F82" s="1">
+        <v>-10.933299999999999</v>
+      </c>
+      <c r="G82" s="1">
+        <v>-37.033299999999997</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
         <v>254</v>
       </c>
-      <c r="D82" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
+      <c r="B83" t="s">
         <v>255</v>
       </c>
-      <c r="B83" t="s">
+      <c r="C83" t="s">
         <v>256</v>
       </c>
-      <c r="C83" t="s">
-        <v>257</v>
-      </c>
       <c r="D83" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F83" s="1">
+        <v>-26.217361</v>
+      </c>
+      <c r="G83" s="1">
+        <v>-48.500971</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>43</v>
       </c>
       <c r="B84" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C84" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D84" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F84" s="1">
+        <v>-26.217361</v>
+      </c>
+      <c r="G84" s="1">
+        <v>-48.500971</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>87</v>
       </c>
       <c r="B85" t="s">
+        <v>258</v>
+      </c>
+      <c r="C85" t="s">
         <v>259</v>
       </c>
-      <c r="C85" t="s">
-        <v>260</v>
-      </c>
       <c r="D85" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F85" s="1">
+        <v>-12.824644773438401</v>
+      </c>
+      <c r="G85" s="1">
+        <v>-38.498511091537601</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>62</v>
       </c>
       <c r="B86" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+      <c r="E86" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F86" s="1">
+        <v>-12.786388000000001</v>
+      </c>
+      <c r="G86" s="1">
+        <v>-38.476944000000003</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>42</v>
       </c>
       <c r="B87" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+      <c r="E87" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F87" s="1">
+        <v>-12.861943999999999</v>
+      </c>
+      <c r="G87" s="1">
+        <v>-38.836111000000002</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>32</v>
       </c>
       <c r="B88" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+      <c r="E88" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F88" s="1">
+        <v>-13.01027777777778</v>
+      </c>
+      <c r="G88" s="1">
+        <v>-38.583333333333343</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>15</v>
       </c>
       <c r="B89" t="s">
+        <v>263</v>
+      </c>
+      <c r="C89" t="s">
         <v>264</v>
       </c>
-      <c r="C89" t="s">
+      <c r="D89" t="s">
         <v>265</v>
       </c>
-      <c r="D89" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E89" t="s">
+        <v>330</v>
+      </c>
+      <c r="F89" s="1">
+        <v>-23.809992999999999</v>
+      </c>
+      <c r="G89" s="1">
+        <v>-45.398988000000003</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>8</v>
       </c>
       <c r="B90" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C90" t="s">
+        <v>264</v>
+      </c>
+      <c r="D90" t="s">
         <v>265</v>
       </c>
-      <c r="D90" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E90" t="s">
+        <v>330</v>
+      </c>
+      <c r="F90" s="1">
+        <v>-23.809992999999999</v>
+      </c>
+      <c r="G90" s="1">
+        <v>-45.398988000000003</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>0</v>
       </c>
       <c r="B91" t="s">
+        <v>267</v>
+      </c>
+      <c r="C91" t="s">
         <v>268</v>
       </c>
-      <c r="C91" t="s">
+      <c r="D91" t="s">
+        <v>265</v>
+      </c>
+      <c r="E91" t="s">
+        <v>330</v>
+      </c>
+      <c r="F91" s="1">
+        <v>-23.956666666666671</v>
+      </c>
+      <c r="G91" s="1">
+        <v>-46.30833333333333</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
         <v>269</v>
       </c>
-      <c r="D91" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
+      <c r="B92" t="s">
         <v>270</v>
       </c>
-      <c r="B92" t="s">
+      <c r="C92" t="s">
         <v>271</v>
-      </c>
-      <c r="C92" t="s">
-        <v>272</v>
       </c>
       <c r="D92" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E92" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F92" s="1">
+        <v>-2.4263880000000002</v>
+      </c>
+      <c r="G92" s="1">
+        <v>-54.694443</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>65</v>
       </c>
       <c r="B93" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C93" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D93" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E93" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F93" s="1">
+        <v>-2.4139569999999999</v>
+      </c>
+      <c r="G93" s="1">
+        <v>-54.738168999999999</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>11</v>
       </c>
       <c r="B94" t="s">
+        <v>273</v>
+      </c>
+      <c r="C94" t="s">
         <v>274</v>
       </c>
-      <c r="C94" t="s">
-        <v>275</v>
-      </c>
       <c r="D94" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+        <v>240</v>
+      </c>
+      <c r="E94" t="s">
+        <v>327</v>
+      </c>
+      <c r="F94" s="1">
+        <v>-8.3941111111111102</v>
+      </c>
+      <c r="G94" s="1">
+        <v>-34.959972222222227</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>40</v>
       </c>
       <c r="B95" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C95" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D95" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E95" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F95" s="1">
+        <v>-1.460277</v>
+      </c>
+      <c r="G95" s="1">
+        <v>-56.380277</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>30</v>
       </c>
       <c r="B96" t="s">
+        <v>276</v>
+      </c>
+      <c r="C96" t="s">
         <v>277</v>
       </c>
-      <c r="C96" t="s">
-        <v>278</v>
-      </c>
       <c r="D96" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E96" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F96" s="1">
+        <v>-29.976666999999999</v>
+      </c>
+      <c r="G96" s="1">
+        <v>-50.123333000000002</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>71</v>
       </c>
       <c r="B97" t="s">
+        <v>278</v>
+      </c>
+      <c r="C97" t="s">
         <v>279</v>
-      </c>
-      <c r="C97" t="s">
-        <v>280</v>
       </c>
       <c r="D97" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E97" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F97" s="1">
+        <v>-1.5694440000000001</v>
+      </c>
+      <c r="G97" s="1">
+        <v>-48.781666000000001</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>63</v>
       </c>
       <c r="B98" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D98" s="1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E98" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F98" s="1">
+        <v>-1.50301530379387</v>
+      </c>
+      <c r="G98" s="1">
+        <v>-48.723792610928903</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
+        <v>281</v>
+      </c>
+      <c r="B99" t="s">
         <v>282</v>
       </c>
-      <c r="B99" t="s">
-        <v>283</v>
-      </c>
       <c r="C99" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D99" s="1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E99" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F99" s="1">
+        <v>-1.505833</v>
+      </c>
+      <c r="G99" s="1">
+        <v>-48.736944000000001</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>28</v>
       </c>
       <c r="B100" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D100" s="1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E100" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F100" s="1">
+        <v>-1.543666666666667</v>
+      </c>
+      <c r="G100" s="1">
+        <v>-48.746499999999997</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>77</v>
       </c>
       <c r="B101" t="s">
+        <v>284</v>
+      </c>
+      <c r="C101" t="s">
         <v>285</v>
       </c>
-      <c r="C101" t="s">
-        <v>286</v>
-      </c>
       <c r="D101" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+        <v>236</v>
+      </c>
+      <c r="E101" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F101" s="1">
+        <v>-20.323889000000001</v>
+      </c>
+      <c r="G101" s="1">
+        <v>-40.321389000000003</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>52</v>
       </c>
       <c r="B102" t="s">
+        <v>286</v>
+      </c>
+      <c r="C102" t="s">
         <v>287</v>
       </c>
-      <c r="C102" t="s">
-        <v>288</v>
-      </c>
       <c r="D102" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+        <v>236</v>
+      </c>
+      <c r="E102" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F102" s="1">
+        <v>-20.288056000000001</v>
+      </c>
+      <c r="G102" s="1">
+        <v>-40.248888000000001</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>17</v>
       </c>
       <c r="B103" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+        <v>236</v>
+      </c>
+      <c r="E103" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F103" s="1">
+        <v>-20.296389000000001</v>
+      </c>
+      <c r="G103" s="1">
+        <v>-40.233333000000002</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>51</v>
       </c>
       <c r="B104" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+        <v>236</v>
+      </c>
+      <c r="E104" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F104" s="1">
+        <v>-20.296389000000001</v>
+      </c>
+      <c r="G104" s="1">
+        <v>-40.233333000000002</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>18</v>
       </c>
       <c r="B105" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+        <v>236</v>
+      </c>
+      <c r="E105" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F105" s="1">
+        <v>-20.258333</v>
+      </c>
+      <c r="G105" s="1">
+        <v>-40.221111000000001</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>48</v>
       </c>
       <c r="B106" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+        <v>236</v>
+      </c>
+      <c r="E106" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F106" s="1">
+        <v>-19.840831999999999</v>
+      </c>
+      <c r="G106" s="1">
+        <v>-40.057499</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>46</v>
       </c>
       <c r="B107" t="s">
+        <v>292</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="D107" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="E107" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F107" s="1">
+        <v>-20.288056000000001</v>
+      </c>
+      <c r="G107" s="1">
+        <v>-40.248888000000001</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
         <v>293</v>
       </c>
-      <c r="C107" s="1" t="s">
-        <v>288</v>
-      </c>
-      <c r="D107" s="1" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
+      <c r="B108" t="s">
         <v>294</v>
       </c>
-      <c r="B108" t="s">
-        <v>295</v>
-      </c>
       <c r="C108" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+        <v>236</v>
+      </c>
+      <c r="E108" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F108" s="1">
+        <v>-20.320277000000001</v>
+      </c>
+      <c r="G108" s="1">
+        <v>-40.305554999999998</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>86</v>
       </c>
       <c r="B109" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C109" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="D109" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="D109" s="1" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E109" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F109" s="1">
+        <v>-19.862500000000001</v>
+      </c>
+      <c r="G109" s="1">
+        <v>-40.070276999999997</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>44</v>
       </c>
       <c r="B110" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+        <v>236</v>
+      </c>
+      <c r="E110" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F110" s="1">
+        <v>-20.321667000000001</v>
+      </c>
+      <c r="G110" s="1">
+        <v>-40.336666999999998</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>68</v>
       </c>
       <c r="B111" t="s">
+        <v>297</v>
+      </c>
+      <c r="C111" t="s">
+        <v>102</v>
+      </c>
+      <c r="D111" t="s">
+        <v>103</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F111" s="1">
+        <v>-4.8736110000000004</v>
+      </c>
+      <c r="G111" s="1">
+        <v>-36.374166000000002</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
         <v>298</v>
       </c>
-      <c r="C111" t="s">
-        <v>103</v>
-      </c>
-      <c r="D111" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
+      <c r="B112" t="s">
         <v>299</v>
       </c>
-      <c r="B112" t="s">
+      <c r="C112" t="s">
+        <v>108</v>
+      </c>
+      <c r="D112" t="s">
+        <v>109</v>
+      </c>
+      <c r="E112" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F112" s="1">
+        <v>-21.868887999999998</v>
+      </c>
+      <c r="G112" s="1">
+        <v>-41.013888000000001</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
         <v>300</v>
       </c>
-      <c r="C112" t="s">
-        <v>109</v>
-      </c>
-      <c r="D112" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
+      <c r="B113" t="s">
         <v>301</v>
       </c>
-      <c r="B113" t="s">
+      <c r="C113" t="s">
+        <v>130</v>
+      </c>
+      <c r="D113" t="s">
+        <v>112</v>
+      </c>
+      <c r="E113" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F113" s="1">
+        <v>-12.783333000000001</v>
+      </c>
+      <c r="G113" s="1">
+        <v>-38.5</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
         <v>302</v>
       </c>
-      <c r="C113" t="s">
-        <v>131</v>
-      </c>
-      <c r="D113" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
+      <c r="B114" t="s">
         <v>303</v>
       </c>
-      <c r="B114" t="s">
-        <v>304</v>
-      </c>
       <c r="C114" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D114" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E114" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F114" s="1">
+        <v>-1.3561110000000001</v>
+      </c>
+      <c r="G114" s="1">
+        <v>-48.481389</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
+        <v>304</v>
+      </c>
+      <c r="B115" t="s">
         <v>305</v>
       </c>
-      <c r="B115" t="s">
+      <c r="C115" t="s">
+        <v>227</v>
+      </c>
+      <c r="D115" t="s">
+        <v>99</v>
+      </c>
+      <c r="E115" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F115" s="1">
+        <v>-29.948609999999999</v>
+      </c>
+      <c r="G115" s="1">
+        <v>-51.623888000000008</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
         <v>306</v>
       </c>
-      <c r="C115" t="s">
-        <v>228</v>
-      </c>
-      <c r="D115" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
+      <c r="B116" t="s">
         <v>307</v>
       </c>
-      <c r="B116" t="s">
+      <c r="C116" t="s">
         <v>308</v>
       </c>
-      <c r="C116" t="s">
+      <c r="D116" t="s">
+        <v>109</v>
+      </c>
+      <c r="E116" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F116" s="1">
+        <v>-22.973333</v>
+      </c>
+      <c r="G116" s="1">
+        <v>-42.013333000000003</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
         <v>309</v>
       </c>
-      <c r="D116" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
+      <c r="B117" t="s">
         <v>310</v>
       </c>
-      <c r="B117" t="s">
+      <c r="C117" t="s">
+        <v>187</v>
+      </c>
+      <c r="D117" t="s">
+        <v>167</v>
+      </c>
+      <c r="E117" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F117" s="1">
+        <v>-3.16</v>
+      </c>
+      <c r="G117" s="1">
+        <v>-59.991109999999999</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
         <v>311</v>
       </c>
-      <c r="C117" t="s">
-        <v>188</v>
-      </c>
-      <c r="D117" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
+      <c r="B118" t="s">
         <v>312</v>
       </c>
-      <c r="B118" t="s">
-        <v>313</v>
-      </c>
       <c r="C118" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D118" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+      <c r="E118" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F118" s="1">
+        <v>-3.1569440000000002</v>
+      </c>
+      <c r="G118" s="1">
+        <v>-59.998609999999992</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>75</v>
       </c>
       <c r="B119" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C119" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D119" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="E119" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F119" s="1">
+        <v>-23.979465992547802</v>
+      </c>
+      <c r="G119" s="1">
+        <v>-46.285389148385001</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>85</v>
       </c>
       <c r="B120" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C120" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D120" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E120" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F120" s="1">
+        <v>-0.85830700000000004</v>
+      </c>
+      <c r="G120" s="1">
+        <v>-52.541353000000001</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
+        <v>315</v>
+      </c>
+      <c r="B121" t="s">
         <v>316</v>
       </c>
-      <c r="B121" t="s">
-        <v>317</v>
-      </c>
       <c r="C121" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D121" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="E121" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F121" s="1">
+        <v>-29.967915999999999</v>
+      </c>
+      <c r="G121" s="1">
+        <v>-51.203611000000002</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>89</v>
       </c>
       <c r="B122" t="s">
+        <v>317</v>
+      </c>
+      <c r="C122" t="s">
+        <v>121</v>
+      </c>
+      <c r="D122" t="s">
+        <v>122</v>
+      </c>
+      <c r="E122" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="F122" s="1">
+        <v>-10.843889000000001</v>
+      </c>
+      <c r="G122" s="1">
+        <v>-36.919167000000002</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
         <v>318</v>
       </c>
-      <c r="C122" t="s">
-        <v>122</v>
-      </c>
-      <c r="D122" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
+      <c r="B123" t="s">
         <v>319</v>
       </c>
-      <c r="B123" t="s">
-        <v>320</v>
-      </c>
       <c r="C123" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D123" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="E123" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F123" s="1">
+        <v>-26.217361</v>
+      </c>
+      <c r="G123" s="1">
+        <v>-48.500971</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>39</v>
       </c>
       <c r="B124" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C124" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D124" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E124" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F124" s="1">
+        <v>-1.4961100000000001</v>
+      </c>
+      <c r="G124" s="1">
+        <v>-48.727221</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
+        <v>321</v>
+      </c>
+      <c r="B125" t="s">
         <v>322</v>
       </c>
-      <c r="B125" t="s">
+      <c r="C125" t="s">
         <v>323</v>
       </c>
-      <c r="C125" t="s">
+      <c r="D125" t="s">
+        <v>142</v>
+      </c>
+      <c r="E125" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F125" s="1">
+        <v>-28.497205999999998</v>
+      </c>
+      <c r="G125" s="1">
+        <v>-48.768999999999998</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
         <v>324</v>
       </c>
-      <c r="D125" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
+      <c r="B126" t="s">
         <v>325</v>
       </c>
-      <c r="B126" t="s">
+      <c r="C126" t="s">
         <v>326</v>
       </c>
-      <c r="C126" t="s">
+      <c r="D126" t="s">
+        <v>112</v>
+      </c>
+      <c r="E126" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="D126" t="s">
-        <v>113</v>
+      <c r="F126" s="1">
+        <v>-17.751387999999999</v>
+      </c>
+      <c r="G126" s="1">
+        <v>-39.216388000000002</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D126" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="A1:G126" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>

</xml_diff>